<commit_message>
Fix PO number extraction to prevent placeholder 'see' from overriding valid PO number
</commit_message>
<xml_diff>
--- a/output/YASKAWA_NEW_SHIPMENT.xlsx
+++ b/output/YASKAWA_NEW_SHIPMENT.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="O2" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P2" s="53" t="n">
@@ -903,7 +903,7 @@
       </c>
       <c r="O3" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P3" s="53" t="n">
@@ -969,7 +969,7 @@
       </c>
       <c r="O4" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P4" s="53" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="O5" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P5" s="53" t="n">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="O6" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P6" s="53" t="n">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="O7" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P7" s="53" t="n">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="O8" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P8" s="53" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="O9" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P9" s="53" t="n">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="O10" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P10" s="53" t="n">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="O11" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P11" s="53" t="n">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="O12" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P12" s="53" t="n">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="O13" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P13" s="53" t="n">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="O14" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P14" s="53" t="n">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="O15" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P15" s="53" t="n">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="O16" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P16" s="53" t="n">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="O17" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P17" s="53" t="n">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="O18" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P18" s="53" t="n">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="O19" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P19" s="53" t="n">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="O20" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P20" s="53" t="n">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="O21" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P21" s="53" t="n">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="O22" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P22" s="53" t="n">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="O23" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P23" s="53" t="n">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="O24" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P24" s="53" t="n">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="O25" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P25" s="53" t="n">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="O26" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P26" s="53" t="n">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="O27" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P27" s="53" t="n">
@@ -2461,7 +2461,7 @@
       </c>
       <c r="O28" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P28" s="53" t="n">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="O29" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P29" s="53" t="n">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="O30" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P30" s="53" t="n">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="O31" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P31" s="53" t="n">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="O32" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P32" s="53" t="n">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="O33" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P33" s="53" t="n">
@@ -2833,7 +2833,7 @@
       </c>
       <c r="O34" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P34" s="53" t="n">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="O35" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P35" s="53" t="n">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="O36" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P36" s="53" t="n">
@@ -3019,7 +3019,7 @@
       </c>
       <c r="O37" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P37" s="53" t="n">
@@ -3081,7 +3081,7 @@
       </c>
       <c r="O38" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P38" s="53" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="O39" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P39" s="53" t="n">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="O40" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P40" s="53" t="n">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="O41" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P41" s="53" t="n">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="O42" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P42" s="53" t="n">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="O43" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P43" s="53" t="n">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="O44" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P44" s="53" t="n">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="O45" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P45" s="53" t="n">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="O46" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P46" s="53" t="n">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="O47" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P47" s="53" t="n">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="O48" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P48" s="53" t="n">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="O49" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P49" s="53" t="n">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="O50" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P50" s="53" t="n">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="O51" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P51" s="53" t="n">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="O52" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P52" s="53" t="n">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="O53" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P53" s="53" t="n">
@@ -4073,7 +4073,7 @@
       </c>
       <c r="O54" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P54" s="53" t="n">
@@ -4135,7 +4135,7 @@
       </c>
       <c r="O55" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P55" s="53" t="n">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="O56" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P56" s="53" t="n">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="O57" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P57" s="53" t="n">
@@ -4321,7 +4321,7 @@
       </c>
       <c r="O58" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P58" s="53" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="O59" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P59" s="53" t="n">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="O60" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P60" s="53" t="n">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="O61" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P61" s="53" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="O62" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P62" s="53" t="n">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="O63" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P63" s="53" t="n">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="O64" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P64" s="53" t="n">
@@ -4755,7 +4755,7 @@
       </c>
       <c r="O65" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P65" s="53" t="n">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="O66" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P66" s="53" t="n">
@@ -4879,7 +4879,7 @@
       </c>
       <c r="O67" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P67" s="53" t="n">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="O68" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P68" s="53" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="O69" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P69" s="53" t="n">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="O70" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P70" s="53" t="n">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="O71" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P71" s="53" t="n">
@@ -5189,7 +5189,7 @@
       </c>
       <c r="O72" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P72" s="53" t="n">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="O73" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P73" s="53" t="n">
@@ -5313,7 +5313,7 @@
       </c>
       <c r="O74" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P74" s="53" t="n">
@@ -5375,7 +5375,7 @@
       </c>
       <c r="O75" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P75" s="53" t="n">
@@ -5437,7 +5437,7 @@
       </c>
       <c r="O76" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P76" s="53" t="n">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="O77" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P77" s="53" t="n">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="O78" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P78" s="53" t="n">
@@ -5623,7 +5623,7 @@
       </c>
       <c r="O79" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P79" s="53" t="n">
@@ -5685,7 +5685,7 @@
       </c>
       <c r="O80" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P80" s="53" t="n">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="O81" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P81" s="53" t="n">
@@ -5809,7 +5809,7 @@
       </c>
       <c r="O82" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P82" s="53" t="n">
@@ -5871,7 +5871,7 @@
       </c>
       <c r="O83" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P83" s="53" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="O84" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P84" s="53" t="n">
@@ -5995,7 +5995,7 @@
       </c>
       <c r="O85" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P85" s="53" t="n">
@@ -6057,7 +6057,7 @@
       </c>
       <c r="O86" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P86" s="53" t="n">
@@ -6119,7 +6119,7 @@
       </c>
       <c r="O87" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P87" s="53" t="n">
@@ -6181,7 +6181,7 @@
       </c>
       <c r="O88" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P88" s="53" t="n">
@@ -6243,7 +6243,7 @@
       </c>
       <c r="O89" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P89" s="53" t="n">
@@ -6305,7 +6305,7 @@
       </c>
       <c r="O90" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P90" s="53" t="n">
@@ -6367,7 +6367,7 @@
       </c>
       <c r="O91" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P91" s="53" t="n">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="O92" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P92" s="53" t="n">
@@ -6491,7 +6491,7 @@
       </c>
       <c r="O93" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P93" s="53" t="n">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="O94" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P94" s="53" t="n">
@@ -6615,7 +6615,7 @@
       </c>
       <c r="O95" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P95" s="53" t="n">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="O96" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P96" s="53" t="n">
@@ -6739,7 +6739,7 @@
       </c>
       <c r="O97" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P97" s="53" t="n">
@@ -6801,7 +6801,7 @@
       </c>
       <c r="O98" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P98" s="53" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="O99" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P99" s="53" t="n">
@@ -6925,7 +6925,7 @@
       </c>
       <c r="O100" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P100" s="53" t="n">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="O101" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P101" s="53" t="n">
@@ -7049,7 +7049,7 @@
       </c>
       <c r="O102" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P102" s="53" t="n">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="O103" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P103" s="53" t="n">
@@ -7173,7 +7173,7 @@
       </c>
       <c r="O104" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P104" s="53" t="n">
@@ -7235,7 +7235,7 @@
       </c>
       <c r="O105" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P105" s="53" t="n">
@@ -7297,7 +7297,7 @@
       </c>
       <c r="O106" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P106" s="53" t="n">
@@ -7359,7 +7359,7 @@
       </c>
       <c r="O107" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P107" s="53" t="n">
@@ -7421,7 +7421,7 @@
       </c>
       <c r="O108" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P108" s="53" t="n">
@@ -7483,7 +7483,7 @@
       </c>
       <c r="O109" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P109" s="53" t="n">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="O110" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P110" s="53" t="n">
@@ -7607,7 +7607,7 @@
       </c>
       <c r="O111" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P111" s="53" t="n">
@@ -7669,7 +7669,7 @@
       </c>
       <c r="O112" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P112" s="53" t="n">
@@ -7731,7 +7731,7 @@
       </c>
       <c r="O113" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P113" s="53" t="n">
@@ -7793,7 +7793,7 @@
       </c>
       <c r="O114" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P114" s="53" t="n">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="O115" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P115" s="53" t="n">
@@ -7917,7 +7917,7 @@
       </c>
       <c r="O116" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P116" s="53" t="n">
@@ -7979,7 +7979,7 @@
       </c>
       <c r="O117" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P117" s="53" t="n">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="O118" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P118" s="53" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="O119" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P119" s="53" t="n">
@@ -8165,7 +8165,7 @@
       </c>
       <c r="O120" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P120" s="53" t="n">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="O121" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P121" s="53" t="n">
@@ -8289,7 +8289,7 @@
       </c>
       <c r="O122" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P122" s="53" t="n">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="O123" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P123" s="53" t="n">
@@ -8413,7 +8413,7 @@
       </c>
       <c r="O124" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P124" s="53" t="n">
@@ -8475,7 +8475,7 @@
       </c>
       <c r="O125" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P125" s="53" t="n">
@@ -8537,7 +8537,7 @@
       </c>
       <c r="O126" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P126" s="53" t="n">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="O127" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P127" s="53" t="n">
@@ -8661,7 +8661,7 @@
       </c>
       <c r="O128" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P128" s="53" t="n">
@@ -8723,7 +8723,7 @@
       </c>
       <c r="O129" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P129" s="53" t="n">
@@ -8785,7 +8785,7 @@
       </c>
       <c r="O130" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P130" s="53" t="n">
@@ -8847,7 +8847,7 @@
       </c>
       <c r="O131" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P131" s="53" t="n">
@@ -8909,7 +8909,7 @@
       </c>
       <c r="O132" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P132" s="53" t="n">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="O133" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P133" s="53" t="n">
@@ -9033,7 +9033,7 @@
       </c>
       <c r="O134" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P134" s="53" t="n">
@@ -9095,7 +9095,7 @@
       </c>
       <c r="O135" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P135" s="53" t="n">
@@ -9157,7 +9157,7 @@
       </c>
       <c r="O136" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P136" s="53" t="n">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="O137" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P137" s="53" t="n">
@@ -9281,7 +9281,7 @@
       </c>
       <c r="O138" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P138" s="53" t="n">
@@ -9343,7 +9343,7 @@
       </c>
       <c r="O139" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P139" s="53" t="n">
@@ -9405,7 +9405,7 @@
       </c>
       <c r="O140" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P140" s="53" t="n">
@@ -9467,7 +9467,7 @@
       </c>
       <c r="O141" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P141" s="53" t="n">
@@ -9529,7 +9529,7 @@
       </c>
       <c r="O142" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P142" s="53" t="n">
@@ -9591,7 +9591,7 @@
       </c>
       <c r="O143" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P143" s="53" t="n">
@@ -9653,7 +9653,7 @@
       </c>
       <c r="O144" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P144" s="53" t="n">
@@ -9715,7 +9715,7 @@
       </c>
       <c r="O145" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P145" s="53" t="n">
@@ -9777,7 +9777,7 @@
       </c>
       <c r="O146" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P146" s="53" t="n">
@@ -9839,7 +9839,7 @@
       </c>
       <c r="O147" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P147" s="53" t="n">
@@ -9901,7 +9901,7 @@
       </c>
       <c r="O148" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P148" s="53" t="n">
@@ -9963,7 +9963,7 @@
       </c>
       <c r="O149" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P149" s="53" t="n">
@@ -10025,7 +10025,7 @@
       </c>
       <c r="O150" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P150" s="53" t="n">
@@ -10087,7 +10087,7 @@
       </c>
       <c r="O151" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P151" s="53" t="n">
@@ -10149,7 +10149,7 @@
       </c>
       <c r="O152" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P152" s="53" t="n">
@@ -10211,7 +10211,7 @@
       </c>
       <c r="O153" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P153" s="53" t="n">
@@ -10273,7 +10273,7 @@
       </c>
       <c r="O154" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P154" s="53" t="n">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="O155" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P155" s="53" t="n">
@@ -10397,7 +10397,7 @@
       </c>
       <c r="O156" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P156" s="53" t="n">
@@ -10459,7 +10459,7 @@
       </c>
       <c r="O157" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P157" s="53" t="n">
@@ -10521,7 +10521,7 @@
       </c>
       <c r="O158" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P158" s="53" t="n">
@@ -10583,7 +10583,7 @@
       </c>
       <c r="O159" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P159" s="53" t="n">
@@ -10645,7 +10645,7 @@
       </c>
       <c r="O160" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P160" s="53" t="n">
@@ -10707,7 +10707,7 @@
       </c>
       <c r="O161" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P161" s="53" t="n">
@@ -10769,7 +10769,7 @@
       </c>
       <c r="O162" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P162" s="53" t="n">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="O163" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P163" s="53" t="n">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="O164" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P164" s="53" t="n">
@@ -10955,7 +10955,7 @@
       </c>
       <c r="O165" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P165" s="53" t="n">
@@ -11017,7 +11017,7 @@
       </c>
       <c r="O166" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P166" s="53" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="O167" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P167" s="53" t="n">
@@ -11141,7 +11141,7 @@
       </c>
       <c r="O168" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P168" s="53" t="n">
@@ -11203,7 +11203,7 @@
       </c>
       <c r="O169" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P169" s="53" t="n">
@@ -11265,7 +11265,7 @@
       </c>
       <c r="O170" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P170" s="53" t="n">
@@ -11327,7 +11327,7 @@
       </c>
       <c r="O171" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P171" s="53" t="n">
@@ -11389,7 +11389,7 @@
       </c>
       <c r="O172" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P172" s="53" t="n">
@@ -11451,7 +11451,7 @@
       </c>
       <c r="O173" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P173" s="53" t="n">
@@ -11513,7 +11513,7 @@
       </c>
       <c r="O174" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P174" s="53" t="n">
@@ -11575,7 +11575,7 @@
       </c>
       <c r="O175" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P175" s="53" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="O176" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P176" s="53" t="n">
@@ -11699,7 +11699,7 @@
       </c>
       <c r="O177" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P177" s="53" t="n">
@@ -11761,7 +11761,7 @@
       </c>
       <c r="O178" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P178" s="53" t="n">
@@ -11823,7 +11823,7 @@
       </c>
       <c r="O179" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P179" s="53" t="n">
@@ -11885,7 +11885,7 @@
       </c>
       <c r="O180" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P180" s="53" t="n">
@@ -11947,7 +11947,7 @@
       </c>
       <c r="O181" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P181" s="53" t="n">
@@ -12009,7 +12009,7 @@
       </c>
       <c r="O182" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P182" s="53" t="n">
@@ -12071,7 +12071,7 @@
       </c>
       <c r="O183" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P183" s="53" t="n">
@@ -12133,7 +12133,7 @@
       </c>
       <c r="O184" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P184" s="53" t="n">
@@ -12195,7 +12195,7 @@
       </c>
       <c r="O185" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P185" s="53" t="n">
@@ -12257,7 +12257,7 @@
       </c>
       <c r="O186" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P186" s="53" t="n">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="O187" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P187" s="53" t="n">
@@ -12381,7 +12381,7 @@
       </c>
       <c r="O188" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P188" s="53" t="n">
@@ -12443,7 +12443,7 @@
       </c>
       <c r="O189" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P189" s="53" t="n">
@@ -12505,7 +12505,7 @@
       </c>
       <c r="O190" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
       <c r="P190" s="53" t="n">
@@ -12567,7 +12567,7 @@
       </c>
       <c r="O191" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P191" s="53" t="n">
@@ -12629,7 +12629,7 @@
       </c>
       <c r="O192" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P192" s="53" t="n">
@@ -12691,7 +12691,7 @@
       </c>
       <c r="O193" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P193" s="53" t="n">
@@ -12753,7 +12753,7 @@
       </c>
       <c r="O194" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P194" s="53" t="n">
@@ -12815,7 +12815,7 @@
       </c>
       <c r="O195" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P195" s="53" t="n">
@@ -12877,7 +12877,7 @@
       </c>
       <c r="O196" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P196" s="53" t="n">
@@ -12939,7 +12939,7 @@
       </c>
       <c r="O197" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P197" s="53" t="n">
@@ -13001,7 +13001,7 @@
       </c>
       <c r="O198" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P198" s="53" t="n">
@@ -13063,7 +13063,7 @@
       </c>
       <c r="O199" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P199" s="53" t="n">
@@ -13125,7 +13125,7 @@
       </c>
       <c r="O200" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P200" s="53" t="n">
@@ -13187,7 +13187,7 @@
       </c>
       <c r="O201" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P201" s="53" t="n">
@@ -13249,7 +13249,7 @@
       </c>
       <c r="O202" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P202" s="53" t="n">
@@ -13311,7 +13311,7 @@
       </c>
       <c r="O203" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P203" s="53" t="n">
@@ -13373,7 +13373,7 @@
       </c>
       <c r="O204" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P204" s="53" t="n">
@@ -13435,7 +13435,7 @@
       </c>
       <c r="O205" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P205" s="53" t="n">
@@ -13497,7 +13497,7 @@
       </c>
       <c r="O206" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P206" s="53" t="n">
@@ -13559,7 +13559,7 @@
       </c>
       <c r="O207" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P207" s="53" t="n">
@@ -13621,7 +13621,7 @@
       </c>
       <c r="O208" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P208" s="53" t="n">
@@ -13683,7 +13683,7 @@
       </c>
       <c r="O209" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P209" s="53" t="n">
@@ -13745,7 +13745,7 @@
       </c>
       <c r="O210" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P210" s="53" t="n">
@@ -13807,7 +13807,7 @@
       </c>
       <c r="O211" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P211" s="53" t="n">
@@ -13869,7 +13869,7 @@
       </c>
       <c r="O212" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P212" s="53" t="n">
@@ -13931,7 +13931,7 @@
       </c>
       <c r="O213" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P213" s="53" t="n">
@@ -13993,7 +13993,7 @@
       </c>
       <c r="O214" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P214" s="53" t="n">
@@ -14055,7 +14055,7 @@
       </c>
       <c r="O215" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P215" s="53" t="n">
@@ -14117,7 +14117,7 @@
       </c>
       <c r="O216" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P216" s="53" t="n">
@@ -14179,7 +14179,7 @@
       </c>
       <c r="O217" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P217" s="53" t="n">
@@ -14241,7 +14241,7 @@
       </c>
       <c r="O218" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P218" s="53" t="n">
@@ -14303,7 +14303,7 @@
       </c>
       <c r="O219" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P219" s="53" t="n">
@@ -14365,7 +14365,7 @@
       </c>
       <c r="O220" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P220" s="53" t="n">
@@ -14427,7 +14427,7 @@
       </c>
       <c r="O221" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P221" s="53" t="n">
@@ -14489,7 +14489,7 @@
       </c>
       <c r="O222" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P222" s="53" t="n">
@@ -14551,7 +14551,7 @@
       </c>
       <c r="O223" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P223" s="53" t="n">
@@ -14613,7 +14613,7 @@
       </c>
       <c r="O224" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P224" s="53" t="n">
@@ -14675,7 +14675,7 @@
       </c>
       <c r="O225" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P225" s="53" t="n">
@@ -14737,7 +14737,7 @@
       </c>
       <c r="O226" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P226" s="53" t="n">
@@ -14799,7 +14799,7 @@
       </c>
       <c r="O227" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P227" s="53" t="n">
@@ -14865,7 +14865,7 @@
       </c>
       <c r="O228" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P228" s="53" t="n">
@@ -14931,7 +14931,7 @@
       </c>
       <c r="O229" s="54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
       <c r="P229" s="53" t="n">
@@ -39543,7 +39543,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39560,7 +39560,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39581,7 +39581,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39602,7 +39602,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39619,7 +39619,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39636,7 +39636,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39653,7 +39653,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39670,7 +39670,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39687,7 +39687,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39704,7 +39704,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39721,7 +39721,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39738,7 +39738,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39755,7 +39755,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39772,7 +39772,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39789,7 +39789,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39806,7 +39806,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39823,7 +39823,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39840,7 +39840,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39857,7 +39857,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39874,7 +39874,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39891,7 +39891,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39908,7 +39908,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39925,7 +39925,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39942,7 +39942,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39959,7 +39959,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39976,7 +39976,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -39993,7 +39993,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40010,7 +40010,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40027,7 +40027,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40044,7 +40044,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40061,7 +40061,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40078,7 +40078,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40095,7 +40095,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40112,7 +40112,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40129,7 +40129,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40146,7 +40146,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40163,7 +40163,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40180,7 +40180,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40197,7 +40197,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40214,7 +40214,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40231,7 +40231,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40248,7 +40248,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40265,7 +40265,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40282,7 +40282,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40299,7 +40299,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40316,7 +40316,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40333,7 +40333,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40350,7 +40350,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40367,7 +40367,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40384,7 +40384,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40401,7 +40401,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40418,7 +40418,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40435,7 +40435,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40452,7 +40452,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40469,7 +40469,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40486,7 +40486,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40503,7 +40503,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40520,7 +40520,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40537,7 +40537,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40554,7 +40554,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40571,7 +40571,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40588,7 +40588,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40605,7 +40605,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40622,7 +40622,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40639,7 +40639,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40656,7 +40656,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40673,7 +40673,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40690,7 +40690,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40707,7 +40707,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40724,7 +40724,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40741,7 +40741,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40758,7 +40758,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40775,7 +40775,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40792,7 +40792,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40809,7 +40809,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40826,7 +40826,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40843,7 +40843,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40860,7 +40860,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40877,7 +40877,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40894,7 +40894,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40911,7 +40911,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40928,7 +40928,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40945,7 +40945,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40962,7 +40962,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40979,7 +40979,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -40996,7 +40996,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41013,7 +41013,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41030,7 +41030,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41047,7 +41047,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41064,7 +41064,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41081,7 +41081,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41098,7 +41098,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41115,7 +41115,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41132,7 +41132,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41149,7 +41149,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41166,7 +41166,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41183,7 +41183,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41200,7 +41200,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41217,7 +41217,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41234,7 +41234,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41251,7 +41251,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41268,7 +41268,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41285,7 +41285,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41302,7 +41302,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41319,7 +41319,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41336,7 +41336,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41353,7 +41353,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41370,7 +41370,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41387,7 +41387,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41404,7 +41404,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41421,7 +41421,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41438,7 +41438,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41455,7 +41455,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41472,7 +41472,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41489,7 +41489,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41506,7 +41506,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41523,7 +41523,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41540,7 +41540,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41557,7 +41557,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41574,7 +41574,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41591,7 +41591,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41608,7 +41608,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41625,7 +41625,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41642,7 +41642,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41659,7 +41659,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41676,7 +41676,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41693,7 +41693,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41710,7 +41710,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41727,7 +41727,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41744,7 +41744,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41761,7 +41761,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41778,7 +41778,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41795,7 +41795,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41812,7 +41812,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41829,7 +41829,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41846,7 +41846,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41863,7 +41863,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41880,7 +41880,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41897,7 +41897,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41914,7 +41914,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41931,7 +41931,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41948,7 +41948,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41965,7 +41965,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41982,7 +41982,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -41999,7 +41999,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42016,7 +42016,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42033,7 +42033,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42050,7 +42050,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42067,7 +42067,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42084,7 +42084,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42101,7 +42101,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42118,7 +42118,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42135,7 +42135,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42152,7 +42152,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42169,7 +42169,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42186,7 +42186,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42203,7 +42203,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42220,7 +42220,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42237,7 +42237,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42254,7 +42254,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42271,7 +42271,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42288,7 +42288,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42305,7 +42305,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42322,7 +42322,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42339,7 +42339,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42356,7 +42356,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42373,7 +42373,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42390,7 +42390,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42407,7 +42407,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42424,7 +42424,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42441,7 +42441,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42458,7 +42458,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42475,7 +42475,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42492,7 +42492,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42509,7 +42509,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42526,7 +42526,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42543,7 +42543,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42560,7 +42560,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42577,7 +42577,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42594,7 +42594,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42611,7 +42611,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42628,7 +42628,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42645,7 +42645,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42662,7 +42662,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42679,7 +42679,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42696,7 +42696,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42713,7 +42713,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42730,7 +42730,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42747,7 +42747,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>PO/V/712</t>
         </is>
       </c>
     </row>
@@ -42764,7 +42764,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42781,7 +42781,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42798,7 +42798,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42815,7 +42815,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42832,7 +42832,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42849,7 +42849,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42866,7 +42866,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42883,7 +42883,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42900,7 +42900,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42917,7 +42917,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42934,7 +42934,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42951,7 +42951,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42968,7 +42968,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -42985,7 +42985,7 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43002,7 +43002,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43019,7 +43019,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43036,7 +43036,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43053,7 +43053,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43070,7 +43070,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43087,7 +43087,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43104,7 +43104,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43121,7 +43121,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43138,7 +43138,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43155,7 +43155,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43172,7 +43172,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43189,7 +43189,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43206,7 +43206,7 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43223,7 +43223,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43240,7 +43240,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43257,7 +43257,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43274,7 +43274,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43291,7 +43291,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43308,7 +43308,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43325,7 +43325,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43342,7 +43342,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43359,7 +43359,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43376,7 +43376,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43397,7 +43397,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>
@@ -43418,7 +43418,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>wer</t>
         </is>
       </c>
     </row>

</xml_diff>